<commit_message>
qol: the abilities of summoned monsters say their figure
the abilities of summoned monsters say their figure (the passives their
chance, songs, dances and stances their size), with the labels of the
same skill of a party member; 107 enemy attacks gain it, the power of an
attack keeps its place on the line
</commit_message>
<xml_diff>
--- a/data_tables/qol_rules.xlsx
+++ b/data_tables/qol_rules.xlsx
@@ -2062,7 +2062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2086,6 +2086,11 @@
           <t>Style</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>After_Power</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -2414,6 +2419,386 @@
       <c r="C23" t="inlineStr">
         <is>
           <t>signed_num</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>251</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Double attack rate</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>252</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Triple attack rate</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>259</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Activation rate</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>260</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Activation rate</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>283</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Occurrence rate</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>316</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>211</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Critical rate</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>plus_num_pct</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>216</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>TP recovery</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>129</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>TP recovery</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>218</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>EXP</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>signed_pct</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>202</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Resistance decrease</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>abs_num</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>193</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>All stats</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>signed_pct</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>26</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ATK</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>signed_pct</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>28</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>signed_pct</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>179</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Damage reduction rate</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>abs_pct</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>136</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Power decrease</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>abs_pct</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>88</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Damage vs. unholy</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>signed_pct</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>137</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Targets</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>66</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Pep</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>signed_num</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
qol: every ability of a summon or a guest ally says its figure
every ability of a summon or a guest ally says its figure: the power of
a spell, what a heal multiplies RES by, the turns of a doll, beside the
passives, songs and stances; 666 of 747 abilities carry added data
</commit_message>
<xml_diff>
--- a/data_tables/qol_rules.xlsx
+++ b/data_tables/qol_rules.xlsx
@@ -2062,7 +2062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2091,6 +2091,11 @@
           <t>After_Power</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -2799,6 +2804,76 @@
       <c r="D42" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>1</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Pwr</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>summons</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>103</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Heals RES</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>half_x</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>summons</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>147</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Turns</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>num</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>summons</t>
         </is>
       </c>
     </row>

</xml_diff>